<commit_message>
updated sesntivity related input files
</commit_message>
<xml_diff>
--- a/sensitivity/sensitivity_input.xlsx
+++ b/sensitivity/sensitivity_input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://esait-my.sharepoint.com/personal/ivo_ferreira_esa_int/Documents/NewAthenaE2EPSF_v3/sensitivity/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="40" documentId="11_2B59D2BFD3305ED8FD6B6E115D3088B352998D12" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02F653E3-1325-924D-8AFF-8FD0283E126C}"/>
+  <xr:revisionPtr revIDLastSave="41" documentId="11_2B59D2BFD3305ED8FD6B6E115D3088B352998D12" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{671F0472-4056-4E4F-8128-AA0C984248CC}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>A_eff</t>
   </si>
@@ -53,24 +53,6 @@
   </si>
   <si>
     <t>Fixed Pseudo-Voigt  8"</t>
-  </si>
-  <si>
-    <t>10% Variable Sym Gaussian 8"</t>
-  </si>
-  <si>
-    <t>50% Variable Sym Gaussian 8"</t>
-  </si>
-  <si>
-    <t>10% Variable Asym Gaussian 8" (ratio 7:1)</t>
-  </si>
-  <si>
-    <t>50% Variable Asym Gaussian 8" (ratio 7:1)</t>
-  </si>
-  <si>
-    <t>10% Variable Pseudo-Voigt 8" (alpha 10%)</t>
-  </si>
-  <si>
-    <t>50% Variable Pseudo-Voigt 8" (alpha 10%)</t>
   </si>
   <si>
     <t>7 keV</t>
@@ -441,7 +423,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
@@ -486,7 +468,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
         <v>10</v>
@@ -499,36 +481,6 @@
       </c>
       <c r="E3" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B8" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B9" t="s">
-        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed vignetting implementation to take into account rowtype and energy (using MM level vignetting functions from SPORT). This version is not clean and includes all the debugging code
</commit_message>
<xml_diff>
--- a/sensitivity/sensitivity_input.xlsx
+++ b/sensitivity/sensitivity_input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://esait-my.sharepoint.com/personal/ivo_ferreira_esa_int/Documents/NewAthenaE2EPSF_v3/sensitivity/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="41" documentId="11_2B59D2BFD3305ED8FD6B6E115D3088B352998D12" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{671F0472-4056-4E4F-8128-AA0C984248CC}"/>
+  <xr:revisionPtr revIDLastSave="70" documentId="11_2B59D2BFD3305ED8FD6B6E115D3088B352998D12" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED0FB777-A294-094F-967B-CF9B0301C93D}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,9 +28,6 @@
     <t>MM_PSF</t>
   </si>
   <si>
-    <t>Fixed Sym Gaussian 8"</t>
-  </si>
-  <si>
     <t>Alignment</t>
   </si>
   <si>
@@ -52,10 +49,13 @@
     <t>1 keV</t>
   </si>
   <si>
-    <t>Fixed Pseudo-Voigt  8"</t>
-  </si>
-  <si>
-    <t>7 keV</t>
+    <t>Fixed Sym Gaussian 0.01"</t>
+  </si>
+  <si>
+    <t>10% Variable Pseudo-Voigt 8" (alpha 10%)</t>
+  </si>
+  <si>
+    <t>30% Variable Pseudo-Voigt 8" (alpha 10%)</t>
   </si>
 </sst>
 </file>
@@ -423,7 +423,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
@@ -440,21 +440,21 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>4</v>
-      </c>
       <c r="E1" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
         <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>2</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -467,20 +467,22 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>11</v>
-      </c>
       <c r="B3" t="s">
         <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E3" t="s">
-        <v>7</v>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B4" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>